<commit_message>
[Excel & YAML] Update Swift CSCF v2026 & v2027
Added source file link
</commit_message>
<xml_diff>
--- a/tools/excel/swift/swift-cscf-v2026.xlsx
+++ b/tools/excel/swift/swift-cscf-v2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\swift\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0973C36D-63C1-4527-8515-C6CA1254ACD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C7FEAD-72AE-4F35-94F2-7472EF6EB3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1416" yWindow="588" windowWidth="20280" windowHeight="11796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>description</t>
   </si>
   <si>
-    <t>This document establishes a set of mandatory and advisory security controls for the operating environment of Swift users. Mandatory security controls build on existing guidance and establish a security baseline for the entire user community. Advisory controls are optional best practices that Swift recommends each user to implement in the operating environment. This document must be read in conjunction with the [CSP FAQ](https://www2.swift.com/kb/#/tip/5021823) Knowledge Base article 5021823 which provides additional valuable information.</t>
-  </si>
-  <si>
     <t>copyright</t>
   </si>
   <si>
@@ -471,6 +468,10 @@
   </si>
   <si>
     <t>Architecture A4 (Advisory)</t>
+  </si>
+  <si>
+    <t>This document establishes a set of mandatory and advisory security controls for the operating environment of Swift users. Mandatory security controls build on existing guidance and establish a security baseline for the entire user community. Advisory controls are optional best practices that Swift recommends each user to implement in the operating environment. This document must be read in conjunction with the [CSP FAQ](https://www2.swift.com/kb/#/tip/5021823) Knowledge Base article 5021823 which provides additional valuable information.
+Source: https://www2.swift.com/knowledgecentre/rest/v1/publications/cscf_dd/76.0/CSCF_v2026_202507015.pdf?logDownload=true</t>
   </si>
 </sst>
 </file>
@@ -931,36 +932,36 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
         <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -982,15 +983,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
         <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -998,7 +999,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1017,20 +1018,20 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
         <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1053,10 +1054,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>8</v>
@@ -1068,7 +1069,7 @@
         <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1076,10 +1077,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
         <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1087,129 +1088,129 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
         <v>30</v>
-      </c>
-      <c r="E3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>34</v>
-      </c>
-      <c r="F4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
         <v>36</v>
       </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
       <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
         <v>38</v>
       </c>
-      <c r="E6" t="s">
-        <v>39</v>
-      </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7">
         <v>3</v>
       </c>
       <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
         <v>40</v>
       </c>
-      <c r="E7" t="s">
-        <v>41</v>
-      </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8">
         <v>3</v>
       </c>
       <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
         <v>42</v>
       </c>
-      <c r="E8" t="s">
-        <v>43</v>
-      </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s">
         <v>44</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>45</v>
-      </c>
-      <c r="F9" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" t="s">
         <v>47</v>
       </c>
-      <c r="E10" t="s">
-        <v>48</v>
-      </c>
       <c r="F10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1217,61 +1218,61 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" t="s">
         <v>49</v>
-      </c>
-      <c r="E11" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12">
         <v>3</v>
       </c>
       <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
         <v>51</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13">
         <v>3</v>
       </c>
       <c r="C13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" t="s">
         <v>54</v>
       </c>
-      <c r="E13" t="s">
-        <v>55</v>
-      </c>
       <c r="F13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>3</v>
       </c>
       <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" t="s">
         <v>56</v>
       </c>
-      <c r="E14" t="s">
-        <v>57</v>
-      </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1279,95 +1280,95 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
         <v>58</v>
-      </c>
-      <c r="E15" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>3</v>
       </c>
       <c r="C16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" t="s">
         <v>60</v>
-      </c>
-      <c r="E16" t="s">
-        <v>34</v>
-      </c>
-      <c r="F16" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17">
         <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18">
         <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19">
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20">
         <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1378,196 +1379,196 @@
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
       <c r="C22" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" t="s">
         <v>67</v>
       </c>
-      <c r="E22" t="s">
-        <v>68</v>
-      </c>
       <c r="F22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23">
         <v>2</v>
       </c>
       <c r="C23" t="s">
+        <v>68</v>
+      </c>
+      <c r="E23" t="s">
         <v>69</v>
       </c>
-      <c r="E23" t="s">
-        <v>70</v>
-      </c>
       <c r="F23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <v>2</v>
       </c>
       <c r="C24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" t="s">
         <v>71</v>
       </c>
-      <c r="E24" t="s">
-        <v>72</v>
-      </c>
       <c r="F24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
       <c r="C25" t="s">
+        <v>72</v>
+      </c>
+      <c r="E25" t="s">
         <v>73</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>74</v>
-      </c>
-      <c r="F25" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="2">
         <v>2</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27">
         <v>2</v>
       </c>
       <c r="C27" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" t="s">
         <v>79</v>
       </c>
-      <c r="E27" t="s">
-        <v>80</v>
-      </c>
       <c r="F27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
         <v>81</v>
       </c>
-      <c r="E28" t="s">
-        <v>82</v>
-      </c>
       <c r="F28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B29">
         <v>2</v>
       </c>
       <c r="C29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" t="s">
         <v>83</v>
       </c>
-      <c r="E29" t="s">
-        <v>84</v>
-      </c>
       <c r="F29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30">
         <v>2</v>
       </c>
       <c r="C30" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" t="s">
         <v>85</v>
       </c>
-      <c r="E30" t="s">
-        <v>86</v>
-      </c>
       <c r="F30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31">
         <v>2</v>
       </c>
       <c r="C31" t="s">
+        <v>86</v>
+      </c>
+      <c r="E31" t="s">
         <v>87</v>
       </c>
-      <c r="E31" t="s">
-        <v>88</v>
-      </c>
       <c r="F31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="2">
         <v>2</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -1575,27 +1576,27 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
+        <v>90</v>
+      </c>
+      <c r="D33" t="s">
         <v>91</v>
-      </c>
-      <c r="D33" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34">
         <v>2</v>
       </c>
       <c r="C34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E34" t="s">
         <v>93</v>
       </c>
-      <c r="E34" t="s">
-        <v>94</v>
-      </c>
       <c r="F34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -1603,44 +1604,44 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
+        <v>94</v>
+      </c>
+      <c r="D35" t="s">
         <v>95</v>
-      </c>
-      <c r="D35" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36">
         <v>2</v>
       </c>
       <c r="C36" t="s">
+        <v>96</v>
+      </c>
+      <c r="E36" t="s">
         <v>97</v>
       </c>
-      <c r="E36" t="s">
-        <v>98</v>
-      </c>
       <c r="F36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B37">
         <v>2</v>
       </c>
       <c r="C37" t="s">
+        <v>98</v>
+      </c>
+      <c r="E37" t="s">
         <v>99</v>
       </c>
-      <c r="E37" t="s">
-        <v>100</v>
-      </c>
       <c r="F37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1648,79 +1649,79 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" t="s">
         <v>101</v>
-      </c>
-      <c r="D38" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39">
         <v>2</v>
       </c>
       <c r="C39" t="s">
+        <v>102</v>
+      </c>
+      <c r="E39" t="s">
         <v>103</v>
       </c>
-      <c r="E39" t="s">
-        <v>104</v>
-      </c>
       <c r="F39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B40">
         <v>2</v>
       </c>
       <c r="C40" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" t="s">
         <v>105</v>
       </c>
-      <c r="E40" t="s">
-        <v>106</v>
-      </c>
       <c r="F40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41" s="2">
         <v>2</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B42">
         <v>2</v>
       </c>
       <c r="C42" t="s">
+        <v>108</v>
+      </c>
+      <c r="E42" t="s">
         <v>109</v>
       </c>
-      <c r="E42" t="s">
-        <v>110</v>
-      </c>
       <c r="F42" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1728,96 +1729,96 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" t="s">
         <v>111</v>
-      </c>
-      <c r="D43" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B44">
         <v>2</v>
       </c>
       <c r="C44" t="s">
+        <v>112</v>
+      </c>
+      <c r="E44" t="s">
         <v>113</v>
       </c>
-      <c r="E44" t="s">
-        <v>114</v>
-      </c>
       <c r="F44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45">
         <v>2</v>
       </c>
       <c r="C45" t="s">
+        <v>114</v>
+      </c>
+      <c r="E45" t="s">
         <v>115</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>116</v>
-      </c>
-      <c r="F45" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46">
         <v>2</v>
       </c>
       <c r="C46" t="s">
+        <v>117</v>
+      </c>
+      <c r="E46" t="s">
         <v>118</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>119</v>
-      </c>
-      <c r="F46" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B47">
         <v>2</v>
       </c>
       <c r="C47" t="s">
+        <v>120</v>
+      </c>
+      <c r="E47" t="s">
         <v>121</v>
       </c>
-      <c r="E47" t="s">
-        <v>122</v>
-      </c>
       <c r="F47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B48" s="2">
         <v>2</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1825,80 +1826,80 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
+        <v>124</v>
+      </c>
+      <c r="D49" t="s">
         <v>125</v>
-      </c>
-      <c r="D49" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B50">
         <v>2</v>
       </c>
       <c r="C50" t="s">
+        <v>126</v>
+      </c>
+      <c r="E50" t="s">
         <v>127</v>
       </c>
-      <c r="E50" t="s">
-        <v>128</v>
-      </c>
       <c r="F50" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B51">
         <v>2</v>
       </c>
       <c r="C51" t="s">
+        <v>128</v>
+      </c>
+      <c r="E51" t="s">
         <v>129</v>
       </c>
-      <c r="E51" t="s">
-        <v>130</v>
-      </c>
       <c r="F51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B52" s="2">
         <v>2</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B53" s="2">
         <v>2</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1923,7 +1924,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1931,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1962,66 +1963,66 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" t="s">
         <v>136</v>
-      </c>
-      <c r="B3" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" t="s">
         <v>138</v>
-      </c>
-      <c r="B4" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" t="s">
         <v>140</v>
-      </c>
-      <c r="B5" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" t="s">
         <v>143</v>
-      </c>
-      <c r="B7" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" t="s">
         <v>145</v>
-      </c>
-      <c r="B8" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B9" t="s">
         <v>147</v>
-      </c>
-      <c r="B9" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>